<commit_message>
Jun + July 2026 finalized
</commit_message>
<xml_diff>
--- a/Jun 2026.xlsx
+++ b/Jun 2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/abutalib/Projects/personal-accounting/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{158513E0-8A4A-A64C-99BB-216E660B0A88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{036E873D-EF83-BE4D-A465-A04375CB84B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="19800" xr2:uid="{7E62CB60-3E82-0E48-87C0-051D0E492E72}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17780" xr2:uid="{7E62CB60-3E82-0E48-87C0-051D0E492E72}"/>
   </bookViews>
   <sheets>
     <sheet name="مصاريف الشهر" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="168">
   <si>
     <t>فاتورة الكهرباء</t>
   </si>
@@ -433,9 +433,6 @@
   </si>
   <si>
     <t>الجهة</t>
-  </si>
-  <si>
-    <t>تمارا</t>
   </si>
   <si>
     <t>تابي</t>
@@ -692,13 +689,13 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -1101,14 +1098,14 @@
       <c r="D1" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="E1" s="19" t="s">
+      <c r="E1" s="20" t="s">
         <v>71</v>
       </c>
-      <c r="F1" s="19"/>
-      <c r="G1" s="19" t="s">
+      <c r="F1" s="20"/>
+      <c r="G1" s="20" t="s">
         <v>70</v>
       </c>
-      <c r="H1" s="19"/>
+      <c r="H1" s="20"/>
       <c r="I1" s="4"/>
       <c r="J1" s="3" t="s">
         <v>17</v>
@@ -1177,7 +1174,7 @@
       </c>
       <c r="AA2" s="3">
         <f>SUM(AA7:AA36)</f>
-        <v>26794</v>
+        <v>23930.67</v>
       </c>
       <c r="AB2" s="4"/>
       <c r="AC2" s="3" t="s">
@@ -1227,7 +1224,7 @@
       </c>
       <c r="AD3" s="3">
         <f>AA21-AD2</f>
-        <v>288</v>
+        <v>-908.32999999999993</v>
       </c>
     </row>
     <row r="4" spans="1:32" x14ac:dyDescent="0.3">
@@ -1307,10 +1304,10 @@
       <c r="O6" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="P6" s="18" t="s">
+      <c r="P6" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="Q6" s="18"/>
+      <c r="Q6" s="19"/>
       <c r="R6" s="9"/>
       <c r="U6" s="9"/>
       <c r="X6" s="9"/>
@@ -1385,7 +1382,7 @@
       </c>
       <c r="C8" s="4"/>
       <c r="D8" s="3" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E8" s="3">
         <v>67</v>
@@ -1444,7 +1441,7 @@
       </c>
       <c r="C9" s="4"/>
       <c r="D9" s="3" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E9" s="3">
         <v>108</v>
@@ -1473,7 +1470,7 @@
       <c r="Y9" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AA9" s="20">
+      <c r="AA9" s="18">
         <f>SUM(Z7:Z8)</f>
         <v>2300</v>
       </c>
@@ -1497,7 +1494,7 @@
       </c>
       <c r="C10" s="4"/>
       <c r="D10" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E10" s="3">
         <v>115</v>
@@ -1542,7 +1539,7 @@
       </c>
       <c r="C11" s="4"/>
       <c r="D11" s="3" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E11" s="3">
         <v>128</v>
@@ -1571,7 +1568,7 @@
       <c r="Y11" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="AA11" s="20">
+      <c r="AA11" s="18">
         <v>3000</v>
       </c>
       <c r="AB11" s="4"/>
@@ -1594,7 +1591,7 @@
       </c>
       <c r="C12" s="4"/>
       <c r="D12" s="3" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E12" s="3">
         <v>150</v>
@@ -1621,7 +1618,7 @@
         <v>77</v>
       </c>
       <c r="AE12" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="13" spans="1:32" x14ac:dyDescent="0.3">
@@ -1633,7 +1630,7 @@
       </c>
       <c r="C13" s="4"/>
       <c r="D13" s="3" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="E13" s="3">
         <v>150</v>
@@ -1655,7 +1652,7 @@
       <c r="Y13" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="AA13" s="20">
+      <c r="AA13" s="18">
         <v>1000</v>
       </c>
       <c r="AB13" s="4"/>
@@ -1678,7 +1675,7 @@
       </c>
       <c r="C14" s="4"/>
       <c r="D14" s="3" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="E14" s="3">
         <v>160</v>
@@ -1708,7 +1705,7 @@
       </c>
       <c r="C15" s="4"/>
       <c r="D15" s="3" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F15" s="3">
         <v>166</v>
@@ -1732,7 +1729,7 @@
       </c>
       <c r="Z15" s="3">
         <f>K27</f>
-        <v>1976.33</v>
+        <v>1007</v>
       </c>
       <c r="AB15" s="4"/>
     </row>
@@ -1740,7 +1737,7 @@
       <c r="B16" s="10"/>
       <c r="C16" s="4"/>
       <c r="D16" s="3" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="F16" s="3">
         <v>230</v>
@@ -1770,7 +1767,7 @@
     <row r="17" spans="3:28" x14ac:dyDescent="0.3">
       <c r="C17" s="4"/>
       <c r="D17" s="3" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="F17" s="3">
         <v>250</v>
@@ -1800,7 +1797,7 @@
     <row r="18" spans="3:28" x14ac:dyDescent="0.3">
       <c r="C18" s="4"/>
       <c r="D18" s="3" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="F18" s="3">
         <v>300</v>
@@ -1822,15 +1819,12 @@
       <c r="Y18" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="Z18" s="3">
-        <v>150</v>
-      </c>
       <c r="AB18" s="4"/>
     </row>
     <row r="19" spans="3:28" x14ac:dyDescent="0.3">
       <c r="C19" s="4"/>
       <c r="D19" s="3" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="F19" s="3">
         <v>350</v>
@@ -1852,15 +1846,12 @@
       <c r="Y19" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="Z19" s="3">
-        <v>77</v>
-      </c>
       <c r="AB19" s="4"/>
     </row>
     <row r="20" spans="3:28" x14ac:dyDescent="0.3">
       <c r="C20" s="4"/>
       <c r="D20" s="3" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E20" s="3">
         <v>1200</v>
@@ -1883,7 +1874,7 @@
       <c r="U20" s="4"/>
       <c r="X20" s="4"/>
       <c r="Y20" s="3" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="Z20" s="3">
         <v>128.66999999999999</v>
@@ -1893,7 +1884,7 @@
     <row r="21" spans="3:28" x14ac:dyDescent="0.3">
       <c r="C21" s="4"/>
       <c r="D21" s="3" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F21" s="3">
         <v>400</v>
@@ -1915,16 +1906,16 @@
       <c r="Y21" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="AA21" s="20">
+      <c r="AA21" s="18">
         <f>SUM(Z15:Z20)</f>
-        <v>3332</v>
+        <v>2135.67</v>
       </c>
       <c r="AB21" s="4"/>
     </row>
     <row r="22" spans="3:28" x14ac:dyDescent="0.3">
       <c r="C22" s="4"/>
       <c r="D22" s="3" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="H22" s="3">
         <v>2636.33</v>
@@ -1955,17 +1946,11 @@
       </c>
       <c r="I23" s="4"/>
       <c r="J23" s="3" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="K23" s="17">
-        <f>(الأرصدة!AA2)-1667</f>
-        <v>969.32999999999993</v>
-      </c>
-      <c r="M23" s="3">
-        <v>1667</v>
-      </c>
-      <c r="N23" s="3">
-        <v>-2636.33</v>
+        <f>(الأرصدة!AA2)</f>
+        <v>0</v>
       </c>
       <c r="O23" s="3">
         <f t="shared" si="1"/>
@@ -1977,7 +1962,7 @@
       <c r="Y23" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="AA23" s="20">
+      <c r="AA23" s="18">
         <f>L27</f>
         <v>820</v>
       </c>
@@ -2000,7 +1985,7 @@
     <row r="25" spans="3:28" x14ac:dyDescent="0.3">
       <c r="C25" s="4"/>
       <c r="D25" s="3" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="F25" s="3">
         <v>150</v>
@@ -2012,7 +1997,7 @@
       <c r="Y25" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="AA25" s="20">
+      <c r="AA25" s="18">
         <v>2000</v>
       </c>
       <c r="AB25" s="4"/>
@@ -2020,7 +2005,7 @@
     <row r="26" spans="3:28" x14ac:dyDescent="0.3">
       <c r="C26" s="3"/>
       <c r="D26" s="3" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="F26" s="3">
         <v>850</v>
@@ -2034,7 +2019,7 @@
     <row r="27" spans="3:28" x14ac:dyDescent="0.3">
       <c r="C27" s="3"/>
       <c r="D27" s="3" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="F27" s="3">
         <v>235</v>
@@ -2045,7 +2030,7 @@
       </c>
       <c r="K27" s="3">
         <f>SUM(K7:K26)</f>
-        <v>1976.33</v>
+        <v>1007</v>
       </c>
       <c r="L27" s="3">
         <f>SUM(L7:L25)</f>
@@ -2053,11 +2038,11 @@
       </c>
       <c r="M27" s="3">
         <f>SUM(M7:M25)</f>
-        <v>3285</v>
+        <v>1618</v>
       </c>
       <c r="N27" s="3">
         <f>SUM(N7:N25)</f>
-        <v>-2636.33</v>
+        <v>0</v>
       </c>
       <c r="R27" s="3"/>
       <c r="U27" s="3"/>
@@ -2074,7 +2059,7 @@
     <row r="28" spans="3:28" x14ac:dyDescent="0.3">
       <c r="C28" s="3"/>
       <c r="D28" s="3" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F28" s="3">
         <v>191</v>
@@ -2088,7 +2073,7 @@
     <row r="29" spans="3:28" x14ac:dyDescent="0.3">
       <c r="C29" s="3"/>
       <c r="D29" s="3" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="H29" s="3">
         <v>128.66999999999999</v>
@@ -2100,9 +2085,9 @@
       <c r="Y29" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="AA29" s="20">
+      <c r="AA29" s="18">
         <f>M27</f>
-        <v>3285</v>
+        <v>1618</v>
       </c>
       <c r="AB29" s="3"/>
     </row>
@@ -2117,7 +2102,7 @@
     <row r="31" spans="3:28" ht="46" x14ac:dyDescent="0.3">
       <c r="C31" s="3"/>
       <c r="D31" s="13" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E31" s="3" t="s">
         <v>93</v>
@@ -2141,7 +2126,7 @@
       <c r="Y31" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="AA31" s="20">
+      <c r="AA31" s="18">
         <f>W2</f>
         <v>12440</v>
       </c>
@@ -2202,7 +2187,7 @@
     </row>
     <row r="36" spans="3:28" x14ac:dyDescent="0.3">
       <c r="Y36" s="3" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="AA36" s="16">
         <v>1667</v>
@@ -2269,9 +2254,6 @@
       <c r="Y44" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="Z44" s="3">
-        <v>-72</v>
-      </c>
       <c r="AB44" s="3"/>
     </row>
     <row r="45" spans="3:28" x14ac:dyDescent="0.3">
@@ -2295,7 +2277,7 @@
       </c>
       <c r="AA46" s="3">
         <f>SUM(Z42:Z45)</f>
-        <v>1930</v>
+        <v>2002</v>
       </c>
     </row>
   </sheetData>
@@ -2351,12 +2333,11 @@
     <col min="24" max="24" width="28.83203125" customWidth="1"/>
     <col min="25" max="25" width="10.1640625" bestFit="1" customWidth="1"/>
     <col min="26" max="26" width="0.5" customWidth="1"/>
-    <col min="27" max="27" width="11" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="20" customWidth="1"/>
+    <col min="27" max="27" width="11" customWidth="1"/>
+    <col min="28" max="28" width="17.33203125" bestFit="1" customWidth="1"/>
     <col min="29" max="29" width="8" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="8.83203125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="8.1640625" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="7.33203125" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="31" max="32" width="10.5" bestFit="1" customWidth="1"/>
     <col min="33" max="33" width="8.83203125" bestFit="1" customWidth="1"/>
     <col min="34" max="34" width="0.5" customWidth="1"/>
   </cols>
@@ -2402,7 +2383,7 @@
         <v>110</v>
       </c>
       <c r="X1" s="3" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="Z1" s="4"/>
       <c r="AA1" s="3" t="s">
@@ -2476,25 +2457,25 @@
       <c r="Z2" s="4"/>
       <c r="AA2" s="11">
         <f>SUM(AG6:AG20)</f>
-        <v>2636.33</v>
+        <v>0</v>
       </c>
       <c r="AB2" s="11"/>
       <c r="AC2" s="11"/>
       <c r="AD2" s="3">
         <f>SUM(AD6:AD20)</f>
-        <v>8711</v>
+        <v>499</v>
       </c>
       <c r="AE2" s="3">
         <f>SUM(AE6:AE20)</f>
-        <v>5909.33</v>
+        <v>499</v>
       </c>
       <c r="AF2" s="3">
         <f>SUM(AF6:AF20)</f>
-        <v>2801.67</v>
+        <v>0</v>
       </c>
       <c r="AG2" s="3">
         <f>SUM(AG6:AG20)</f>
-        <v>2636.33</v>
+        <v>0</v>
       </c>
       <c r="AH2" s="4"/>
     </row>
@@ -2683,27 +2664,26 @@
       </c>
       <c r="Z6" s="4"/>
       <c r="AA6" s="3">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AB6" s="3" t="s">
-        <v>128</v>
+        <v>158</v>
       </c>
       <c r="AC6" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="AD6" s="3">
-        <v>1995</v>
+        <v>499</v>
       </c>
       <c r="AE6" s="3">
-        <f>998+499</f>
-        <v>1497</v>
+        <v>499</v>
       </c>
       <c r="AF6" s="3">
         <f>AD6-AE6</f>
-        <v>498</v>
+        <v>0</v>
       </c>
       <c r="AG6" s="3">
-        <v>499</v>
+        <v>0</v>
       </c>
       <c r="AH6" s="4"/>
     </row>
@@ -2765,29 +2745,13 @@
         <v>500</v>
       </c>
       <c r="Z7" s="4"/>
-      <c r="AA7" s="3">
-        <v>4</v>
-      </c>
-      <c r="AB7" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="AC7" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="AD7" s="3">
-        <v>1216</v>
-      </c>
-      <c r="AE7" s="3">
-        <f>608+304</f>
-        <v>912</v>
-      </c>
-      <c r="AF7" s="3">
-        <f>AD7-AE7</f>
-        <v>304</v>
-      </c>
-      <c r="AG7" s="3">
-        <v>304</v>
-      </c>
+      <c r="AA7" s="3"/>
+      <c r="AB7" s="3"/>
+      <c r="AC7" s="3"/>
+      <c r="AD7" s="3"/>
+      <c r="AE7" s="3"/>
+      <c r="AF7" s="3"/>
+      <c r="AG7" s="3"/>
       <c r="AH7" s="4"/>
     </row>
     <row r="8" spans="1:34" ht="22" x14ac:dyDescent="0.3">
@@ -2850,31 +2814,13 @@
         <v>303</v>
       </c>
       <c r="Z8" s="4"/>
-      <c r="AA8" s="3">
-        <v>4</v>
-      </c>
-      <c r="AB8" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="AC8" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="AD8" s="3">
-        <f>AG8*3</f>
-        <v>5001</v>
-      </c>
-      <c r="AE8" s="3">
-        <f>1667*2</f>
-        <v>3334</v>
-      </c>
-      <c r="AF8" s="3">
-        <f>AD8-AE8</f>
-        <v>1667</v>
-      </c>
-      <c r="AG8" s="3">
-        <f>1618+49</f>
-        <v>1667</v>
-      </c>
+      <c r="AA8" s="3"/>
+      <c r="AB8" s="3"/>
+      <c r="AC8" s="3"/>
+      <c r="AD8" s="3"/>
+      <c r="AE8" s="3"/>
+      <c r="AF8" s="3"/>
+      <c r="AG8" s="3"/>
       <c r="AH8" s="4"/>
     </row>
     <row r="9" spans="1:34" ht="22" x14ac:dyDescent="0.3">
@@ -2937,28 +2883,6 @@
         <v>750</v>
       </c>
       <c r="Z9" s="4"/>
-      <c r="AA9" s="3">
-        <v>6</v>
-      </c>
-      <c r="AB9" s="3" t="s">
-        <v>159</v>
-      </c>
-      <c r="AC9" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="AD9" s="3">
-        <v>499</v>
-      </c>
-      <c r="AE9" s="3">
-        <v>166.33</v>
-      </c>
-      <c r="AF9" s="3">
-        <f>AD9-AE9</f>
-        <v>332.66999999999996</v>
-      </c>
-      <c r="AG9" s="3">
-        <v>166.33</v>
-      </c>
       <c r="AH9" s="4"/>
     </row>
     <row r="10" spans="1:34" ht="22" x14ac:dyDescent="0.3">
@@ -3335,7 +3259,7 @@
         <v>4</v>
       </c>
       <c r="X16" s="3" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="Y16" s="11"/>
       <c r="Z16" s="4"/>
@@ -3437,7 +3361,7 @@
         <v>4</v>
       </c>
       <c r="X18" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Y18" s="3">
         <v>228</v>
@@ -3476,7 +3400,7 @@
         <v>5</v>
       </c>
       <c r="T19" s="3" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="U19" s="11">
         <v>3600</v>
@@ -3486,7 +3410,7 @@
         <v>4</v>
       </c>
       <c r="X19" s="3" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="Y19" s="5">
         <v>1957</v>
@@ -3523,7 +3447,7 @@
         <v>6</v>
       </c>
       <c r="T20" s="3" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="U20" s="3">
         <v>2107</v>
@@ -3533,7 +3457,7 @@
         <v>4</v>
       </c>
       <c r="X20" s="3" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="Y20" s="11">
         <v>479</v>
@@ -3570,7 +3494,7 @@
         <v>6</v>
       </c>
       <c r="T21" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="U21" s="3">
         <v>3000</v>
@@ -3607,7 +3531,7 @@
         <v>6</v>
       </c>
       <c r="T22" s="3" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="U22" s="3">
         <v>3680</v>
@@ -3749,7 +3673,7 @@
         <v>97</v>
       </c>
       <c r="AB26" s="3" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="AC26">
         <v>5001</v>
@@ -3856,7 +3780,7 @@
       <c r="I30" s="3"/>
       <c r="J30" s="3"/>
       <c r="L30" s="3" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="M30" s="6">
         <f>M23+M27+M26</f>

</xml_diff>